<commit_message>
Prefactibilidad por consola con PDF
</commit_message>
<xml_diff>
--- a/Program/Datos/datos_manuales.xlsx
+++ b/Program/Datos/datos_manuales.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mhoyosme\Desktop\Proyecto\Program\Datos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C9D62192-68A2-48DB-9119-0E82294732E7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CF89A593-B5FD-42A7-8B6D-5AB7283AC40F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" activeTab="1" xr2:uid="{CD6D87B3-3E85-4D9D-BFF0-D4E802493E81}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="581" uniqueCount="196">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="596" uniqueCount="198">
   <si>
     <t>75.0</t>
   </si>
@@ -627,6 +627,12 @@
   </si>
   <si>
     <t>Fusible PDB2 B</t>
+  </si>
+  <si>
+    <t>AC</t>
+  </si>
+  <si>
+    <t>DC</t>
   </si>
 </sst>
 </file>
@@ -739,34 +745,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="39">
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
-    <dxf>
-      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
-    </dxf>
+  <dxfs count="40">
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
@@ -1146,6 +1125,36 @@
       </fill>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
@@ -1160,64 +1169,65 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5874A6EA-08E4-4C13-B67C-CB816184D3C0}" name="Tabla2" displayName="Tabla2" ref="A1:G2" totalsRowShown="0" headerRowDxfId="38" dataDxfId="36" headerRowBorderDxfId="37" tableBorderDxfId="35" totalsRowBorderDxfId="34">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{5874A6EA-08E4-4C13-B67C-CB816184D3C0}" name="Tabla2" displayName="Tabla2" ref="A1:G2" totalsRowShown="0" headerRowDxfId="29" dataDxfId="27" headerRowBorderDxfId="28" tableBorderDxfId="26" totalsRowBorderDxfId="25">
   <autoFilter ref="A1:G2" xr:uid="{5874A6EA-08E4-4C13-B67C-CB816184D3C0}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{9F2439FA-30A1-4D90-9F47-A866995AD462}" name="nombre_nodo" dataDxfId="33"/>
-    <tableColumn id="5" xr3:uid="{E1FDA295-F988-4715-B9C7-42286712743D}" name="tipo" dataDxfId="32"/>
-    <tableColumn id="6" xr3:uid="{E955F37D-B353-4F7A-9521-F49CF205229C}" name="codigo" dataDxfId="31"/>
-    <tableColumn id="7" xr3:uid="{22F231D9-9879-4122-9BAF-253B8C04BB15}" name="regional" dataDxfId="30"/>
-    <tableColumn id="2" xr3:uid="{CA56A5C1-DCFB-45F9-A91D-E19FDCFDDF4C}" name="direccion" dataDxfId="29"/>
-    <tableColumn id="3" xr3:uid="{42241B89-6C4C-4F8D-8BF0-C33F36C93C1D}" name="capacidad_kva" dataDxfId="28"/>
-    <tableColumn id="4" xr3:uid="{96DBA14E-72BF-4616-A90F-5169ACCA998C}" name="voltaje_sistema_dc" dataDxfId="27"/>
+    <tableColumn id="1" xr3:uid="{9F2439FA-30A1-4D90-9F47-A866995AD462}" name="nombre_nodo" dataDxfId="24"/>
+    <tableColumn id="5" xr3:uid="{E1FDA295-F988-4715-B9C7-42286712743D}" name="tipo" dataDxfId="23"/>
+    <tableColumn id="6" xr3:uid="{E955F37D-B353-4F7A-9521-F49CF205229C}" name="codigo" dataDxfId="22"/>
+    <tableColumn id="7" xr3:uid="{22F231D9-9879-4122-9BAF-253B8C04BB15}" name="regional" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{CA56A5C1-DCFB-45F9-A91D-E19FDCFDDF4C}" name="direccion" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{42241B89-6C4C-4F8D-8BF0-C33F36C93C1D}" name="capacidad_kva" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{96DBA14E-72BF-4616-A90F-5169ACCA998C}" name="voltaje_sistema_dc" dataDxfId="18"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2E5421E9-2724-423C-851B-A0845D404EE3}" name="Tabla3" displayName="Tabla3" ref="A1:F15" totalsRowShown="0" headerRowDxfId="26" dataDxfId="25">
-  <autoFilter ref="A1:F15" xr:uid="{2E5421E9-2724-423C-851B-A0845D404EE3}"/>
-  <tableColumns count="6">
-    <tableColumn id="7" xr3:uid="{4DA03894-7D07-44E5-BB0D-94373ECA9338}" name="ubicacion" dataDxfId="24"/>
-    <tableColumn id="1" xr3:uid="{FEF86DC1-CDF6-4D2B-9711-3CE2E8FDC61D}" name="componente" dataDxfId="23"/>
-    <tableColumn id="2" xr3:uid="{E8898F3B-F793-4C03-9ADB-3E0756FDECAF}" name="marca" dataDxfId="22"/>
-    <tableColumn id="3" xr3:uid="{E4F60FA1-A5C6-4AC3-BF15-A364399D1E4E}" name="referencia" dataDxfId="21"/>
-    <tableColumn id="4" xr3:uid="{CD65DA30-5B1A-4E7C-8023-7B23F0D22BDF}" name="capacidad_amps" dataDxfId="20"/>
-    <tableColumn id="5" xr3:uid="{00B2E6A4-9D0B-4CA9-A4F2-C6F8CCF0A7FC}" name="calibre_cable_awg" dataDxfId="19"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="3" xr:uid="{2E5421E9-2724-423C-851B-A0845D404EE3}" name="Tabla3" displayName="Tabla3" ref="A1:G15" totalsRowShown="0" headerRowDxfId="17" dataDxfId="16">
+  <autoFilter ref="A1:G15" xr:uid="{2E5421E9-2724-423C-851B-A0845D404EE3}"/>
+  <tableColumns count="7">
+    <tableColumn id="7" xr3:uid="{4DA03894-7D07-44E5-BB0D-94373ECA9338}" name="ubicacion" dataDxfId="15"/>
+    <tableColumn id="1" xr3:uid="{FEF86DC1-CDF6-4D2B-9711-3CE2E8FDC61D}" name="componente" dataDxfId="14"/>
+    <tableColumn id="2" xr3:uid="{E8898F3B-F793-4C03-9ADB-3E0756FDECAF}" name="marca" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{E4F60FA1-A5C6-4AC3-BF15-A364399D1E4E}" name="referencia" dataDxfId="12"/>
+    <tableColumn id="4" xr3:uid="{CD65DA30-5B1A-4E7C-8023-7B23F0D22BDF}" name="capacidad_amps" dataDxfId="11"/>
+    <tableColumn id="6" xr3:uid="{EC182694-78B3-42C0-947F-3CB1555CB945}" name="tipo" dataDxfId="0"/>
+    <tableColumn id="5" xr3:uid="{00B2E6A4-9D0B-4CA9-A4F2-C6F8CCF0A7FC}" name="calibre_cable_awg" dataDxfId="10"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F279930-8CE0-4458-A500-A4804307D033}" name="Tabla4" displayName="Tabla4" ref="A1:G95" totalsRowShown="0" headerRowDxfId="18" dataDxfId="17">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{4F279930-8CE0-4458-A500-A4804307D033}" name="Tabla4" displayName="Tabla4" ref="A1:G95" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8">
   <autoFilter ref="A1:G95" xr:uid="{4F279930-8CE0-4458-A500-A4804307D033}"/>
   <tableColumns count="7">
-    <tableColumn id="1" xr3:uid="{6CBBC484-43B4-4212-8A72-72C36A0AA59A}" name="pdb_nombre" dataDxfId="16"/>
-    <tableColumn id="2" xr3:uid="{E0A6FC31-B215-4C57-B8C0-A8E53A5B832B}" name="fuente" dataDxfId="15"/>
-    <tableColumn id="3" xr3:uid="{4F3E6BCE-4115-4327-9F4D-9FE1AB222BE1}" name="posicion" dataDxfId="14"/>
-    <tableColumn id="4" xr3:uid="{0F488469-BA24-4436-842B-6D2F9F8F4214}" name="estado" dataDxfId="13"/>
-    <tableColumn id="5" xr3:uid="{DAED4AB6-F7E7-4C43-9177-F8900C29D95C}" name="capacidad" dataDxfId="12"/>
-    <tableColumn id="7" xr3:uid="{59F7B2D4-6A80-447C-B8ED-E0F301A44C2C}" name="corriente" dataDxfId="11"/>
-    <tableColumn id="6" xr3:uid="{DCE97B5A-FEBD-4BAD-9EB4-7754B346D6AB}" name="equipo_refencia" dataDxfId="10"/>
+    <tableColumn id="1" xr3:uid="{6CBBC484-43B4-4212-8A72-72C36A0AA59A}" name="pdb_nombre" dataDxfId="7"/>
+    <tableColumn id="2" xr3:uid="{E0A6FC31-B215-4C57-B8C0-A8E53A5B832B}" name="fuente" dataDxfId="6"/>
+    <tableColumn id="3" xr3:uid="{4F3E6BCE-4115-4327-9F4D-9FE1AB222BE1}" name="posicion" dataDxfId="5"/>
+    <tableColumn id="4" xr3:uid="{0F488469-BA24-4436-842B-6D2F9F8F4214}" name="estado" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{DAED4AB6-F7E7-4C43-9177-F8900C29D95C}" name="capacidad" dataDxfId="3"/>
+    <tableColumn id="7" xr3:uid="{59F7B2D4-6A80-447C-B8ED-E0F301A44C2C}" name="corriente" dataDxfId="2"/>
+    <tableColumn id="6" xr3:uid="{DCE97B5A-FEBD-4BAD-9EB4-7754B346D6AB}" name="equipo_refencia" dataDxfId="1"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DE2280A1-9E4C-4DCD-BF7E-888FBA537ECA}" name="Tabla1" displayName="Tabla1" ref="A1:H13" totalsRowShown="0" headerRowDxfId="9" dataDxfId="8" headerRowCellStyle="Normal" dataCellStyle="Normal">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{DE2280A1-9E4C-4DCD-BF7E-888FBA537ECA}" name="Tabla1" displayName="Tabla1" ref="A1:H13" totalsRowShown="0" headerRowDxfId="39" dataDxfId="38" headerRowCellStyle="Normal" dataCellStyle="Normal">
   <autoFilter ref="A1:H13" xr:uid="{DE2280A1-9E4C-4DCD-BF7E-888FBA537ECA}"/>
   <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{3AB90701-9B35-41AA-99FD-EA000C0FBAC6}" name="nombre_rack" dataDxfId="7" dataCellStyle="Normal"/>
-    <tableColumn id="10" xr3:uid="{552625CA-FFA9-4D0F-9AE4-8E8AA2CFD81A}" name="Label" dataDxfId="6" dataCellStyle="Normal"/>
-    <tableColumn id="4" xr3:uid="{4E5A4E54-6DE7-48C8-8A66-7C97E2FA04A1}" name="u_totales" dataDxfId="5" dataCellStyle="Normal"/>
-    <tableColumn id="11" xr3:uid="{BE625927-AF15-478E-87C9-1BC144738D1C}" name="Espacio" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{D32C66C7-BCD4-4610-8774-1CC22DE4F9A0}" name="u_ocupadas_listado" dataDxfId="3" dataCellStyle="Normal"/>
-    <tableColumn id="6" xr3:uid="{282C4EE8-ED53-4C8B-B914-B33DF7A75E4D}" name="u_libres_listado" dataDxfId="2" dataCellStyle="Normal"/>
-    <tableColumn id="7" xr3:uid="{D325EA4D-3855-4FB8-8337-3E9BBFFDA68B}" name="nombre_foto" dataDxfId="1" dataCellStyle="Normal"/>
-    <tableColumn id="8" xr3:uid="{94BF02C2-1F70-4B1B-94F9-F73DDBFA1E1A}" name="Detalle_rack" dataDxfId="0" dataCellStyle="Normal"/>
+    <tableColumn id="1" xr3:uid="{3AB90701-9B35-41AA-99FD-EA000C0FBAC6}" name="nombre_rack" dataDxfId="37" dataCellStyle="Normal"/>
+    <tableColumn id="10" xr3:uid="{552625CA-FFA9-4D0F-9AE4-8E8AA2CFD81A}" name="Label" dataDxfId="36" dataCellStyle="Normal"/>
+    <tableColumn id="4" xr3:uid="{4E5A4E54-6DE7-48C8-8A66-7C97E2FA04A1}" name="u_totales" dataDxfId="35" dataCellStyle="Normal"/>
+    <tableColumn id="11" xr3:uid="{BE625927-AF15-478E-87C9-1BC144738D1C}" name="Espacio" dataDxfId="34"/>
+    <tableColumn id="5" xr3:uid="{D32C66C7-BCD4-4610-8774-1CC22DE4F9A0}" name="u_ocupadas_listado" dataDxfId="33" dataCellStyle="Normal"/>
+    <tableColumn id="6" xr3:uid="{282C4EE8-ED53-4C8B-B914-B33DF7A75E4D}" name="u_libres_listado" dataDxfId="32" dataCellStyle="Normal"/>
+    <tableColumn id="7" xr3:uid="{D325EA4D-3855-4FB8-8337-3E9BBFFDA68B}" name="nombre_foto" dataDxfId="31" dataCellStyle="Normal"/>
+    <tableColumn id="8" xr3:uid="{94BF02C2-1F70-4B1B-94F9-F73DDBFA1E1A}" name="Detalle_rack" dataDxfId="30" dataCellStyle="Normal"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1607,7 +1617,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70FE85F0-6249-49C0-98C3-75140ABDEF17}">
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="24.85546875" customWidth="1"/>
@@ -1618,7 +1628,7 @@
     <col min="6" max="6" width="22.28515625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>99</v>
       </c>
@@ -1635,10 +1645,13 @@
         <v>92</v>
       </c>
       <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
         <v>180</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>82</v>
       </c>
@@ -1655,10 +1668,13 @@
         <v>200</v>
       </c>
       <c r="F2" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G2" s="1" t="s">
         <v>181</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>82</v>
       </c>
@@ -1674,11 +1690,14 @@
       <c r="E3" s="1">
         <v>400</v>
       </c>
-      <c r="F3" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F3" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G3" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>82</v>
       </c>
@@ -1694,11 +1713,14 @@
       <c r="E4" s="1">
         <v>400</v>
       </c>
-      <c r="F4" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F4" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G4" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>81</v>
       </c>
@@ -1714,13 +1736,16 @@
       <c r="E5" s="1">
         <v>225</v>
       </c>
-      <c r="F5" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F5" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G5" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>19</v>
@@ -1735,12 +1760,15 @@
         <v>125</v>
       </c>
       <c r="F6" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>20</v>
@@ -1755,10 +1783,13 @@
         <v>125</v>
       </c>
       <c r="F7" s="1" t="s">
+        <v>196</v>
+      </c>
+      <c r="G7" s="1" t="s">
         <v>182</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>83</v>
       </c>
@@ -1774,11 +1805,14 @@
       <c r="E8" s="1">
         <v>500</v>
       </c>
-      <c r="F8" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F8" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G8" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A9" s="1" t="s">
         <v>83</v>
       </c>
@@ -1794,11 +1828,14 @@
       <c r="E9" s="1">
         <v>500</v>
       </c>
-      <c r="F9" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F9" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G9" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
         <v>84</v>
       </c>
@@ -1814,11 +1851,14 @@
       <c r="E10" s="1">
         <v>500</v>
       </c>
-      <c r="F10" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F10" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
         <v>84</v>
       </c>
@@ -1834,11 +1874,14 @@
       <c r="E11" s="1">
         <v>500</v>
       </c>
-      <c r="F11" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F11" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G11" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
         <v>24</v>
       </c>
@@ -1854,11 +1897,14 @@
       <c r="E12" s="1">
         <v>150</v>
       </c>
-      <c r="F12" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F12" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G12" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A13" s="1" t="s">
         <v>24</v>
       </c>
@@ -1874,11 +1920,14 @@
       <c r="E13" s="1">
         <v>150</v>
       </c>
-      <c r="F13" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F13" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G13" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>23</v>
       </c>
@@ -1894,11 +1943,14 @@
       <c r="E14" s="1">
         <v>250</v>
       </c>
-      <c r="F14" s="1">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.25">
+      <c r="F14" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G14" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="1" t="s">
         <v>23</v>
       </c>
@@ -1914,7 +1966,10 @@
       <c r="E15" s="1">
         <v>250</v>
       </c>
-      <c r="F15" s="1">
+      <c r="F15" s="1" t="s">
+        <v>197</v>
+      </c>
+      <c r="G15" s="1">
         <v>0</v>
       </c>
     </row>

</xml_diff>